<commit_message>
Bump bay costs to full-premium spec in the Phase 1 budget
Ahead of the county DEI meeting and landlord conversations, moved the
Budget column to match the existing Full Premium column for every
SIMULATOR EQUIPMENT and BAY CONSTRUCTION line item in
Fairway_Golf_Club_Phase1_Budget_200K.xlsx (projectors, screens,
enclosures, PCs, side monitors, framing, acoustic treatment, turf,
electrical, HVAC, divider wall, LED lighting) -- the actual golf
technology and bay build now reflect a stronger, more credible spec
for an external audience, while lounge/reception/beverage/signage/soft
costs stay value-engineered.

New Phase 1 Investment: $170,060 (was $135,630), still under the
$200K target. Updated the now-stale "smart swap" notes on the affected
rows so they don't contradict the new premium figures. Refreshed
CLAUDE.md's Open Financial Reconciliation table to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fairway_Golf_Club_Phase1_Budget_200K.xlsx
+++ b/Fairway_Golf_Club_Phase1_Budget_200K.xlsx
@@ -1,25 +1,32 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Budget Summary" sheetId="1" state="visible" r:id="rId3"/>
-  </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Template/>
+  <TotalTime>0</TotalTime>
+  <Application>LibreOffice/26.2.4.2$Linux_AARCH64 LibreOffice_project/620$Build-2</Application>
+  <AppVersion>15.0000</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-07-03T01:03:37Z</dcterms:created>
+  <dc:creator>openpyxl</dc:creator>
+  <dc:description/>
+  <dc:language>en-US</dc:language>
+  <cp:lastModifiedBy/>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-07-03T01:03:37Z</dcterms:modified>
+  <cp:revision>0</cp:revision>
+  <dc:subject/>
+  <dc:title/>
+</cp:coreProperties>
+</file>
+
+<file path=docProps\custom.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes"/>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="115">
   <si>
     <t xml:space="preserve">FAIRWAY GOLF CLUB</t>
@@ -369,7 +376,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
@@ -726,7 +733,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -901,7 +908,27 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="4"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Budget Summary" sheetId="1" state="visible" r:id="rId3"/>
+  </sheets>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001" fullCalcOnLoad="1"/>
+  <extLst>
+    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -968,13 +995,15 @@
         <v>10</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>4000</v>
+        <v>7000</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>7000</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>11</v>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Upgraded to BenQ cinema-grade ($3.5K ea) — full premium spec</t>
+        </is>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -982,13 +1011,15 @@
         <v>12</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>1600</v>
+        <v>3000</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>3000</v>
       </c>
-      <c r="E10" s="10" t="s">
-        <v>13</v>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Upgraded to full premium screens (10,500 ea)</t>
+        </is>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -996,13 +1027,15 @@
         <v>14</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>1200</v>
+        <v>4000</v>
       </c>
       <c r="D11" s="9" t="n">
         <v>4000</v>
       </c>
-      <c r="E11" s="10" t="s">
-        <v>15</v>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Upgraded to pre-fab enclosure frames</t>
+        </is>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1010,13 +1043,15 @@
         <v>16</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>4000</v>
+        <v>6000</v>
       </c>
       <c r="D12" s="9" t="n">
         <v>6000</v>
       </c>
-      <c r="E12" s="10" t="s">
-        <v>17</v>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Upgraded to full premium PC build</t>
+        </is>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1066,13 +1101,15 @@
         <v>24</v>
       </c>
       <c r="C16" s="8" t="n">
-        <v>800</v>
+        <v>1600</v>
       </c>
       <c r="D16" s="9" t="n">
         <v>1600</v>
       </c>
-      <c r="E16" s="10" t="s">
-        <v>25</v>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Upgraded to commercial-grade displays</t>
+        </is>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1085,7 +1122,7 @@
         <v>27</v>
       </c>
       <c r="C19" s="8" t="n">
-        <v>8000</v>
+        <v>12000</v>
       </c>
       <c r="D19" s="9" t="n">
         <v>12000</v>
@@ -1099,13 +1136,15 @@
         <v>29</v>
       </c>
       <c r="C20" s="8" t="n">
-        <v>2400</v>
+        <v>8000</v>
       </c>
       <c r="D20" s="9" t="n">
         <v>8000</v>
       </c>
-      <c r="E20" s="10" t="s">
-        <v>30</v>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>Upgraded to commercial acoustic treatment ($4K/bay)</t>
+        </is>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1113,13 +1152,15 @@
         <v>31</v>
       </c>
       <c r="C21" s="8" t="n">
-        <v>3200</v>
+        <v>5000</v>
       </c>
       <c r="D21" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="E21" s="10" t="s">
-        <v>32</v>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>Upgraded to installed premium turf</t>
+        </is>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1127,7 +1168,7 @@
         <v>33</v>
       </c>
       <c r="C22" s="8" t="n">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="D22" s="9" t="n">
         <v>5000</v>
@@ -1141,7 +1182,7 @@
         <v>35</v>
       </c>
       <c r="C23" s="8" t="n">
-        <v>5000</v>
+        <v>8000</v>
       </c>
       <c r="D23" s="9" t="n">
         <v>8000</v>
@@ -1155,7 +1196,7 @@
         <v>37</v>
       </c>
       <c r="C24" s="8" t="n">
-        <v>4000</v>
+        <v>6000</v>
       </c>
       <c r="D24" s="9" t="n">
         <v>6000</v>
@@ -1169,7 +1210,7 @@
         <v>39</v>
       </c>
       <c r="C25" s="8" t="n">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="D25" s="9" t="n">
         <v>3000</v>
@@ -1183,13 +1224,15 @@
         <v>41</v>
       </c>
       <c r="C26" s="8" t="n">
-        <v>600</v>
+        <v>2000</v>
       </c>
       <c r="D26" s="9" t="n">
         <v>2000</v>
       </c>
-      <c r="E26" s="10" t="s">
-        <v>42</v>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>Upgraded to custom LED installation</t>
+        </is>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1658,7 +1701,7 @@
       </c>
       <c r="C70" s="13" t="n">
         <f aca="false">SUM(C8,C9,C10,C11,C12,C13,C14,C15,C16,C19,C20,C21,C22,C23,C24,C25,C26,C29,C30,C31,C32,C33,C34,C35,C36,C37,C38,C39,C40,C43,C44,C45,C46,C47,C50,C51,C52,C53,C54,C55,C58,C59,C60,C63,C64,C65,C66,C67)</f>
-        <v>123300</v>
+        <v>154600</v>
       </c>
       <c r="D70" s="14" t="n">
         <f aca="false">SUM(D8,D9,D10,D11,D12,D13,D14,D15,D16,D19,D20,D21,D22,D23,D24,D25,D26,D29,D30,D31,D32,D33,D34,D35,D36,D37,D38,D39,D40,D43,D44,D45,D46,D47,D50,D51,D52,D53,D54,D55,D58,D59,D60,D63,D64,D65,D66,D67)</f>
@@ -1671,7 +1714,7 @@
       </c>
       <c r="C71" s="16" t="n">
         <f aca="false">C70*0.1</f>
-        <v>12330</v>
+        <v>15460</v>
       </c>
       <c r="D71" s="14" t="n">
         <f aca="false">D70*0.1</f>
@@ -1684,7 +1727,7 @@
       </c>
       <c r="C72" s="18" t="n">
         <f aca="false">C70+C71</f>
-        <v>135630</v>
+        <v>170060</v>
       </c>
       <c r="D72" s="19" t="n">
         <f aca="false">D70+D71</f>
@@ -1698,7 +1741,7 @@
       </c>
       <c r="C73" s="21" t="n">
         <f aca="false">D72-C72</f>
-        <v>131230</v>
+        <v>96800</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>